<commit_message>
fix: template limpio sin comentarios + visor con navegacion horizontal
- Eliminados comentarios del template (comments1.xml, vmlDrawing,
  referencias en rels y content types)
- ResultView ahora muestra pares debito/credito (OutputRow[])
- Navegacion horizontal por grupos de columnas (6 paginas)
- Botones Anterior/Siguiente + indicadores de pagina
- El Excel generado ya no hereda comentarios del template
</commit_message>
<xml_diff>
--- a/public/Modelodeimportacion.xlsx
+++ b/public/Modelodeimportacion.xlsx
@@ -35,525 +35,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Andres Felipe Ruiz Velasco</author>
-    <author>Deimer Esteban Peña Gonzalez</author>
-    <author>Ivan Dario Corchuelo Castro</author>
-    <author>deimer esteban peña gonzalez</author>
-    <author>Cristian Andres Collazos Ruiz</author>
-    <author>David Felipe Penagos Mosquera</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>*Campo obligatorio
-*Campo numérico, 3 caracteres
-Digita el código del tipo del comprobante contable
-Eje: 1 , 121, 999 
-Importante
-Repetir el código dependiendo de la cantidad de  item</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>*Campo obligatorio
-Digitar el consecutivo del comprobante contable
-Ejemplo: 10</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>*Campo obligatorio
-*Formato de DD/MM/AAAA</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Este campo es obligatorio en caso de manejar moneda extranjera
-Ejemplo:
-- COP
-- USD</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0000-000005000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">* Campo numérico de 5 enteros y 9 decimales
-* Este campo será obligatorio al tener una moneda diferente a la local y debe ser mayor a cero
-* La tasa puede estar en una sola secuencia o en todas, pero no puede tener dos tasas diferentes para el comprobante
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000006000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Campo obligatorio
-* Digitar código a nivel transaccional</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="3" shapeId="0" xr:uid="{00000000-0006-0000-0000-000007000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>*Campo obligatorio
-Digitar el número de identificación sin digito de verificación</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000008000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>*Digite sucursal solo si el tercero tiene, caso contrario deje en blanco 
-* Campo numérico de 3 caracteres</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000009000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si la cuenta contable esta asociada a un grupo de inventario, este campo será obligatorio</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="3" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000A000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si la cuenta contable esta asociada a un grupo de inventario, este campo será obligatorio
-*Aplica solo si tiene manejo de bodegas y si producto maneja control de inventarios</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="4" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000B000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">* Si la cuenta contable esta asociada a un grupo de inventario, este campo será obligatorio.
-Se debe adicionar el signo + o - </t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000C000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si la cuenta contable esta asociada a un grupo de inventario, este campo será obligatorio</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000D000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si la cuenta contable maneja vencimiento cartera o proveedor, este campo será obligatorio
-* Campo alfanumérico, permite  - , .  
-* Máximo 6 Caracteres</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000E000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si cuenta contable maneja vencimiento cartera o proveedor, este campo será obligatorio</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-00000F000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si la cuenta contable maneja vencimiento cartera o proveedor, este campo será obligatorio
-* Máximo 3 caracteres</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000010000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si la cuenta contable maneja vencimiento cartera o proveedor, este campo será obligatorio
-*Formato de DD/MM/AAAA</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000011000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si la cuenta contable esta asociada a un impuesto, este campo será obligatorio</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R1" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0000-000012000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si la cuenta contable esta asociada un grupo de activos, este campo será obligatorio</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000013000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Si la cuenta contable esta asociada un grupo de activos, este campo será obligatorio</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000014000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Campo alfanumérico
-* Máximo 100 caracteres</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="3" shapeId="0" xr:uid="{00000000-0006-0000-0000-000015000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Digita el código del centro-subcentro, según la ruta Configuración - transacciones - centro de costo. 
-Ejemplo 1-1  </t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve"> </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="2" shapeId="0" xr:uid="{00000000-0006-0000-0000-000016000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Campo numérico, 11 enteros 2 decimales</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000017000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Campo numérico, 11 enteros 2 decimales</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000018000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Campo alfanumérico
-* Máximo 300 caracteres</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-000019000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Campo numérico, 11 enteros 2 decimales
-* Digita si el comprobante hace base  para libro de ventas o de compras</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="1" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001A000000}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>* Campo numérico, 11 enteros 2 decimales
-* Digita  si el comprobante hace base  para libro de ventas o de compras</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA1" authorId="5" shapeId="0" xr:uid="{00000000-0006-0000-0000-00001B000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>David Felipe Penagos Mosquera:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-*Si el comprobante se va a crear en el Mes de cierre del periodo fiscal, especificar con SI o NO</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>